<commit_message>
Strengthen fixtures after review and skip missing Downloads books.
Add a visible Ashery Master tab, real J&M panel-option SKUs, and an
Options tab on the wide_species book. Live Mac-path tests now skip
instead of returning green when the file is absent.

Co-authored-by: Koffeekinggamer <Koffeekinggamer@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/settled/ashery-oak.xlsx
+++ b/tests/fixtures/settled/ashery-oak.xlsx
@@ -10,7 +10,8 @@
     <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Markup" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Options&amp;Portal" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Products" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Master" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Products" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -563,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +649,99 @@
         <v>450</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Oak / Rustic Cherry</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Hickory</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>QSWO / Cherry</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Model #</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Overall Size</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>10% More</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>35% More</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BARN FLOOR OCCASIONAL TABLES</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>BF-1648-END</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>End Table</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>24"W x 16"D x 24"H</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D4" t="n">
         <v>220</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E4" t="n">
         <v>230</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F4" t="n">
         <v>280</v>
       </c>
     </row>

</xml_diff>